<commit_message>
feat: implement strict doctor access control, full web-mobile parity, and closed cases modal
</commit_message>
<xml_diff>
--- a/appium-tests/ReconAI_Appium_E2E_Test_Report_300_TestCases.xlsx
+++ b/appium-tests/ReconAI_Appium_E2E_Test_Report_300_TestCases.xlsx
@@ -17,7 +17,7 @@
     <t>RECONAI MOBILE SURGICAL PLATFORM - APPIUM E2E TEST SUITE REPORT</t>
   </si>
   <si>
-    <t>Execution Date: 11/8/2026 | Platform: Appium 2.x (UiAutomator2 &amp; XCUITest) | Target: ReconAI Mobile Frontend</t>
+    <t>Execution Date: 14/8/2026 | Platform: Appium 2.x (UiAutomator2 &amp; XCUITest) | Target: ReconAI Mobile Frontend</t>
   </si>
   <si>
     <t>1. OVERALL EXECUTION KPI METRICS</t>
@@ -197,7 +197,7 @@
     <t>Android 13.0</t>
   </si>
   <si>
-    <t>2026-08-11T03:33:49.528Z</t>
+    <t>2026-08-14T04:03:04.199Z</t>
   </si>
   <si>
     <t>TC-APP-002</t>
@@ -4097,7 +4097,7 @@
         <v>30</v>
       </c>
       <c r="K2" s="19">
-        <v>342</v>
+        <v>155</v>
       </c>
       <c r="L2" s="16" t="s">
         <v>59</v>
@@ -4138,7 +4138,7 @@
         <v>30</v>
       </c>
       <c r="K3" s="19">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="L3" s="16" t="s">
         <v>59</v>
@@ -4179,7 +4179,7 @@
         <v>32</v>
       </c>
       <c r="K4" s="19">
-        <v>543</v>
+        <v>191</v>
       </c>
       <c r="L4" s="16" t="s">
         <v>59</v>
@@ -4220,7 +4220,7 @@
         <v>32</v>
       </c>
       <c r="K5" s="19">
-        <v>431</v>
+        <v>201</v>
       </c>
       <c r="L5" s="16" t="s">
         <v>59</v>
@@ -4261,7 +4261,7 @@
         <v>34</v>
       </c>
       <c r="K6" s="19">
-        <v>479</v>
+        <v>185</v>
       </c>
       <c r="L6" s="16" t="s">
         <v>81</v>
@@ -4302,7 +4302,7 @@
         <v>34</v>
       </c>
       <c r="K7" s="19">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>81</v>
@@ -4343,7 +4343,7 @@
         <v>34</v>
       </c>
       <c r="K8" s="19">
-        <v>302</v>
+        <v>493</v>
       </c>
       <c r="L8" s="16" t="s">
         <v>59</v>
@@ -4384,7 +4384,7 @@
         <v>32</v>
       </c>
       <c r="K9" s="19">
-        <v>317</v>
+        <v>289</v>
       </c>
       <c r="L9" s="16" t="s">
         <v>59</v>
@@ -4425,7 +4425,7 @@
         <v>30</v>
       </c>
       <c r="K10" s="19">
-        <v>339</v>
+        <v>188</v>
       </c>
       <c r="L10" s="16" t="s">
         <v>59</v>
@@ -4466,7 +4466,7 @@
         <v>34</v>
       </c>
       <c r="K11" s="19">
-        <v>353</v>
+        <v>237</v>
       </c>
       <c r="L11" s="16" t="s">
         <v>81</v>
@@ -4507,7 +4507,7 @@
         <v>32</v>
       </c>
       <c r="K12" s="19">
-        <v>213</v>
+        <v>395</v>
       </c>
       <c r="L12" s="16" t="s">
         <v>59</v>
@@ -4548,7 +4548,7 @@
         <v>34</v>
       </c>
       <c r="K13" s="19">
-        <v>357</v>
+        <v>531</v>
       </c>
       <c r="L13" s="16" t="s">
         <v>59</v>
@@ -4589,7 +4589,7 @@
         <v>30</v>
       </c>
       <c r="K14" s="19">
-        <v>416</v>
+        <v>437</v>
       </c>
       <c r="L14" s="16" t="s">
         <v>59</v>
@@ -4630,7 +4630,7 @@
         <v>32</v>
       </c>
       <c r="K15" s="19">
-        <v>281</v>
+        <v>196</v>
       </c>
       <c r="L15" s="16" t="s">
         <v>81</v>
@@ -4671,7 +4671,7 @@
         <v>30</v>
       </c>
       <c r="K16" s="19">
-        <v>323</v>
+        <v>427</v>
       </c>
       <c r="L16" s="16" t="s">
         <v>59</v>
@@ -4712,7 +4712,7 @@
         <v>30</v>
       </c>
       <c r="K17" s="19">
-        <v>256</v>
+        <v>500</v>
       </c>
       <c r="L17" s="16" t="s">
         <v>59</v>
@@ -4753,7 +4753,7 @@
         <v>30</v>
       </c>
       <c r="K18" s="19">
-        <v>204</v>
+        <v>408</v>
       </c>
       <c r="L18" s="16" t="s">
         <v>59</v>
@@ -4794,7 +4794,7 @@
         <v>32</v>
       </c>
       <c r="K19" s="19">
-        <v>339</v>
+        <v>476</v>
       </c>
       <c r="L19" s="16" t="s">
         <v>59</v>
@@ -4835,7 +4835,7 @@
         <v>32</v>
       </c>
       <c r="K20" s="19">
-        <v>295</v>
+        <v>483</v>
       </c>
       <c r="L20" s="16" t="s">
         <v>59</v>
@@ -4876,7 +4876,7 @@
         <v>34</v>
       </c>
       <c r="K21" s="19">
-        <v>522</v>
+        <v>405</v>
       </c>
       <c r="L21" s="16" t="s">
         <v>81</v>
@@ -4917,7 +4917,7 @@
         <v>34</v>
       </c>
       <c r="K22" s="19">
-        <v>517</v>
+        <v>232</v>
       </c>
       <c r="L22" s="16" t="s">
         <v>81</v>
@@ -4958,7 +4958,7 @@
         <v>34</v>
       </c>
       <c r="K23" s="19">
-        <v>405</v>
+        <v>440</v>
       </c>
       <c r="L23" s="16" t="s">
         <v>59</v>
@@ -4999,7 +4999,7 @@
         <v>32</v>
       </c>
       <c r="K24" s="19">
-        <v>437</v>
+        <v>197</v>
       </c>
       <c r="L24" s="16" t="s">
         <v>59</v>
@@ -5040,7 +5040,7 @@
         <v>30</v>
       </c>
       <c r="K25" s="19">
-        <v>191</v>
+        <v>314</v>
       </c>
       <c r="L25" s="16" t="s">
         <v>59</v>
@@ -5081,7 +5081,7 @@
         <v>34</v>
       </c>
       <c r="K26" s="19">
-        <v>517</v>
+        <v>343</v>
       </c>
       <c r="L26" s="16" t="s">
         <v>81</v>
@@ -5122,7 +5122,7 @@
         <v>32</v>
       </c>
       <c r="K27" s="19">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="L27" s="16" t="s">
         <v>59</v>
@@ -5163,7 +5163,7 @@
         <v>34</v>
       </c>
       <c r="K28" s="19">
-        <v>353</v>
+        <v>501</v>
       </c>
       <c r="L28" s="16" t="s">
         <v>59</v>
@@ -5204,7 +5204,7 @@
         <v>30</v>
       </c>
       <c r="K29" s="19">
-        <v>155</v>
+        <v>242</v>
       </c>
       <c r="L29" s="16" t="s">
         <v>59</v>
@@ -5245,7 +5245,7 @@
         <v>32</v>
       </c>
       <c r="K30" s="19">
-        <v>198</v>
+        <v>379</v>
       </c>
       <c r="L30" s="16" t="s">
         <v>81</v>
@@ -5286,7 +5286,7 @@
         <v>30</v>
       </c>
       <c r="K31" s="19">
-        <v>375</v>
+        <v>219</v>
       </c>
       <c r="L31" s="16" t="s">
         <v>59</v>
@@ -5327,7 +5327,7 @@
         <v>30</v>
       </c>
       <c r="K32" s="19">
-        <v>445</v>
+        <v>516</v>
       </c>
       <c r="L32" s="16" t="s">
         <v>59</v>
@@ -5368,7 +5368,7 @@
         <v>30</v>
       </c>
       <c r="K33" s="19">
-        <v>382</v>
+        <v>496</v>
       </c>
       <c r="L33" s="16" t="s">
         <v>59</v>
@@ -5409,7 +5409,7 @@
         <v>32</v>
       </c>
       <c r="K34" s="19">
-        <v>155</v>
+        <v>274</v>
       </c>
       <c r="L34" s="16" t="s">
         <v>59</v>
@@ -5450,7 +5450,7 @@
         <v>32</v>
       </c>
       <c r="K35" s="19">
-        <v>433</v>
+        <v>306</v>
       </c>
       <c r="L35" s="16" t="s">
         <v>59</v>
@@ -5491,7 +5491,7 @@
         <v>34</v>
       </c>
       <c r="K36" s="19">
-        <v>497</v>
+        <v>169</v>
       </c>
       <c r="L36" s="16" t="s">
         <v>81</v>
@@ -5532,7 +5532,7 @@
         <v>34</v>
       </c>
       <c r="K37" s="19">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="L37" s="16" t="s">
         <v>81</v>
@@ -5573,7 +5573,7 @@
         <v>34</v>
       </c>
       <c r="K38" s="19">
-        <v>350</v>
+        <v>388</v>
       </c>
       <c r="L38" s="16" t="s">
         <v>59</v>
@@ -5614,7 +5614,7 @@
         <v>32</v>
       </c>
       <c r="K39" s="19">
-        <v>317</v>
+        <v>445</v>
       </c>
       <c r="L39" s="16" t="s">
         <v>59</v>
@@ -5655,7 +5655,7 @@
         <v>30</v>
       </c>
       <c r="K40" s="19">
-        <v>161</v>
+        <v>533</v>
       </c>
       <c r="L40" s="16" t="s">
         <v>59</v>
@@ -5696,7 +5696,7 @@
         <v>34</v>
       </c>
       <c r="K41" s="19">
-        <v>364</v>
+        <v>427</v>
       </c>
       <c r="L41" s="16" t="s">
         <v>81</v>
@@ -5737,7 +5737,7 @@
         <v>32</v>
       </c>
       <c r="K42" s="19">
-        <v>494</v>
+        <v>401</v>
       </c>
       <c r="L42" s="16" t="s">
         <v>59</v>
@@ -5778,7 +5778,7 @@
         <v>34</v>
       </c>
       <c r="K43" s="19">
-        <v>169</v>
+        <v>196</v>
       </c>
       <c r="L43" s="16" t="s">
         <v>59</v>
@@ -5819,7 +5819,7 @@
         <v>30</v>
       </c>
       <c r="K44" s="19">
-        <v>502</v>
+        <v>181</v>
       </c>
       <c r="L44" s="16" t="s">
         <v>59</v>
@@ -5860,7 +5860,7 @@
         <v>32</v>
       </c>
       <c r="K45" s="19">
-        <v>463</v>
+        <v>270</v>
       </c>
       <c r="L45" s="16" t="s">
         <v>81</v>
@@ -5901,7 +5901,7 @@
         <v>30</v>
       </c>
       <c r="K46" s="19">
-        <v>379</v>
+        <v>155</v>
       </c>
       <c r="L46" s="16" t="s">
         <v>59</v>
@@ -5942,7 +5942,7 @@
         <v>32</v>
       </c>
       <c r="K47" s="19">
-        <v>465</v>
+        <v>230</v>
       </c>
       <c r="L47" s="16" t="s">
         <v>59</v>
@@ -5983,7 +5983,7 @@
         <v>32</v>
       </c>
       <c r="K48" s="19">
-        <v>160</v>
+        <v>445</v>
       </c>
       <c r="L48" s="16" t="s">
         <v>59</v>
@@ -6024,7 +6024,7 @@
         <v>34</v>
       </c>
       <c r="K49" s="19">
-        <v>200</v>
+        <v>146</v>
       </c>
       <c r="L49" s="16" t="s">
         <v>81</v>
@@ -6065,7 +6065,7 @@
         <v>34</v>
       </c>
       <c r="K50" s="19">
-        <v>120</v>
+        <v>367</v>
       </c>
       <c r="L50" s="16" t="s">
         <v>59</v>
@@ -6106,7 +6106,7 @@
         <v>34</v>
       </c>
       <c r="K51" s="19">
-        <v>127</v>
+        <v>177</v>
       </c>
       <c r="L51" s="16" t="s">
         <v>59</v>
@@ -6147,7 +6147,7 @@
         <v>36</v>
       </c>
       <c r="K52" s="19">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="L52" s="16" t="s">
         <v>81</v>
@@ -6188,7 +6188,7 @@
         <v>32</v>
       </c>
       <c r="K53" s="19">
-        <v>240</v>
+        <v>436</v>
       </c>
       <c r="L53" s="16" t="s">
         <v>59</v>
@@ -6229,7 +6229,7 @@
         <v>30</v>
       </c>
       <c r="K54" s="19">
-        <v>183</v>
+        <v>140</v>
       </c>
       <c r="L54" s="16" t="s">
         <v>59</v>
@@ -6270,7 +6270,7 @@
         <v>34</v>
       </c>
       <c r="K55" s="19">
-        <v>454</v>
+        <v>121</v>
       </c>
       <c r="L55" s="16" t="s">
         <v>59</v>
@@ -6311,7 +6311,7 @@
         <v>32</v>
       </c>
       <c r="K56" s="19">
-        <v>425</v>
+        <v>371</v>
       </c>
       <c r="L56" s="16" t="s">
         <v>59</v>
@@ -6352,7 +6352,7 @@
         <v>36</v>
       </c>
       <c r="K57" s="19">
-        <v>204</v>
+        <v>159</v>
       </c>
       <c r="L57" s="16" t="s">
         <v>81</v>
@@ -6393,7 +6393,7 @@
         <v>30</v>
       </c>
       <c r="K58" s="19">
-        <v>325</v>
+        <v>442</v>
       </c>
       <c r="L58" s="16" t="s">
         <v>59</v>
@@ -6434,7 +6434,7 @@
         <v>34</v>
       </c>
       <c r="K59" s="19">
-        <v>463</v>
+        <v>162</v>
       </c>
       <c r="L59" s="16" t="s">
         <v>59</v>
@@ -6475,7 +6475,7 @@
         <v>36</v>
       </c>
       <c r="K60" s="19">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="L60" s="16" t="s">
         <v>81</v>
@@ -6516,7 +6516,7 @@
         <v>34</v>
       </c>
       <c r="K61" s="19">
-        <v>246</v>
+        <v>312</v>
       </c>
       <c r="L61" s="16" t="s">
         <v>59</v>
@@ -6557,7 +6557,7 @@
         <v>32</v>
       </c>
       <c r="K62" s="19">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="L62" s="16" t="s">
         <v>59</v>
@@ -6598,7 +6598,7 @@
         <v>32</v>
       </c>
       <c r="K63" s="19">
-        <v>264</v>
+        <v>221</v>
       </c>
       <c r="L63" s="16" t="s">
         <v>59</v>
@@ -6639,7 +6639,7 @@
         <v>34</v>
       </c>
       <c r="K64" s="19">
-        <v>261</v>
+        <v>141</v>
       </c>
       <c r="L64" s="16" t="s">
         <v>81</v>
@@ -6680,7 +6680,7 @@
         <v>34</v>
       </c>
       <c r="K65" s="19">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="L65" s="16" t="s">
         <v>59</v>
@@ -6721,7 +6721,7 @@
         <v>34</v>
       </c>
       <c r="K66" s="19">
-        <v>382</v>
+        <v>283</v>
       </c>
       <c r="L66" s="16" t="s">
         <v>59</v>
@@ -6762,7 +6762,7 @@
         <v>36</v>
       </c>
       <c r="K67" s="19">
-        <v>240</v>
+        <v>311</v>
       </c>
       <c r="L67" s="16" t="s">
         <v>81</v>
@@ -6803,7 +6803,7 @@
         <v>32</v>
       </c>
       <c r="K68" s="19">
-        <v>400</v>
+        <v>440</v>
       </c>
       <c r="L68" s="16" t="s">
         <v>59</v>
@@ -6844,7 +6844,7 @@
         <v>30</v>
       </c>
       <c r="K69" s="19">
-        <v>184</v>
+        <v>450</v>
       </c>
       <c r="L69" s="16" t="s">
         <v>59</v>
@@ -6885,7 +6885,7 @@
         <v>34</v>
       </c>
       <c r="K70" s="19">
-        <v>187</v>
+        <v>306</v>
       </c>
       <c r="L70" s="16" t="s">
         <v>59</v>
@@ -6926,7 +6926,7 @@
         <v>32</v>
       </c>
       <c r="K71" s="19">
-        <v>284</v>
+        <v>210</v>
       </c>
       <c r="L71" s="16" t="s">
         <v>59</v>
@@ -6967,7 +6967,7 @@
         <v>36</v>
       </c>
       <c r="K72" s="19">
-        <v>371</v>
+        <v>335</v>
       </c>
       <c r="L72" s="16" t="s">
         <v>81</v>
@@ -7008,7 +7008,7 @@
         <v>30</v>
       </c>
       <c r="K73" s="19">
-        <v>366</v>
+        <v>325</v>
       </c>
       <c r="L73" s="16" t="s">
         <v>59</v>
@@ -7049,7 +7049,7 @@
         <v>34</v>
       </c>
       <c r="K74" s="19">
-        <v>135</v>
+        <v>447</v>
       </c>
       <c r="L74" s="16" t="s">
         <v>59</v>
@@ -7090,7 +7090,7 @@
         <v>36</v>
       </c>
       <c r="K75" s="19">
-        <v>437</v>
+        <v>360</v>
       </c>
       <c r="L75" s="16" t="s">
         <v>81</v>
@@ -7131,7 +7131,7 @@
         <v>34</v>
       </c>
       <c r="K76" s="19">
-        <v>361</v>
+        <v>152</v>
       </c>
       <c r="L76" s="16" t="s">
         <v>59</v>
@@ -7172,7 +7172,7 @@
         <v>32</v>
       </c>
       <c r="K77" s="19">
-        <v>269</v>
+        <v>364</v>
       </c>
       <c r="L77" s="16" t="s">
         <v>59</v>
@@ -7213,7 +7213,7 @@
         <v>32</v>
       </c>
       <c r="K78" s="19">
-        <v>435</v>
+        <v>395</v>
       </c>
       <c r="L78" s="16" t="s">
         <v>59</v>
@@ -7254,7 +7254,7 @@
         <v>34</v>
       </c>
       <c r="K79" s="19">
-        <v>433</v>
+        <v>142</v>
       </c>
       <c r="L79" s="16" t="s">
         <v>81</v>
@@ -7295,7 +7295,7 @@
         <v>34</v>
       </c>
       <c r="K80" s="19">
-        <v>461</v>
+        <v>146</v>
       </c>
       <c r="L80" s="16" t="s">
         <v>59</v>
@@ -7336,7 +7336,7 @@
         <v>34</v>
       </c>
       <c r="K81" s="19">
-        <v>333</v>
+        <v>377</v>
       </c>
       <c r="L81" s="16" t="s">
         <v>59</v>
@@ -7377,7 +7377,7 @@
         <v>36</v>
       </c>
       <c r="K82" s="19">
-        <v>379</v>
+        <v>338</v>
       </c>
       <c r="L82" s="16" t="s">
         <v>81</v>
@@ -7418,7 +7418,7 @@
         <v>32</v>
       </c>
       <c r="K83" s="19">
-        <v>376</v>
+        <v>357</v>
       </c>
       <c r="L83" s="16" t="s">
         <v>59</v>
@@ -7459,7 +7459,7 @@
         <v>30</v>
       </c>
       <c r="K84" s="19">
-        <v>288</v>
+        <v>362</v>
       </c>
       <c r="L84" s="16" t="s">
         <v>59</v>
@@ -7500,7 +7500,7 @@
         <v>34</v>
       </c>
       <c r="K85" s="19">
-        <v>339</v>
+        <v>181</v>
       </c>
       <c r="L85" s="16" t="s">
         <v>59</v>
@@ -7541,7 +7541,7 @@
         <v>32</v>
       </c>
       <c r="K86" s="19">
-        <v>132</v>
+        <v>444</v>
       </c>
       <c r="L86" s="16" t="s">
         <v>59</v>
@@ -7582,7 +7582,7 @@
         <v>36</v>
       </c>
       <c r="K87" s="19">
-        <v>370</v>
+        <v>434</v>
       </c>
       <c r="L87" s="16" t="s">
         <v>81</v>
@@ -7623,7 +7623,7 @@
         <v>30</v>
       </c>
       <c r="K88" s="19">
-        <v>312</v>
+        <v>435</v>
       </c>
       <c r="L88" s="16" t="s">
         <v>59</v>
@@ -7664,7 +7664,7 @@
         <v>34</v>
       </c>
       <c r="K89" s="19">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="L89" s="16" t="s">
         <v>59</v>
@@ -7705,7 +7705,7 @@
         <v>36</v>
       </c>
       <c r="K90" s="19">
-        <v>267</v>
+        <v>249</v>
       </c>
       <c r="L90" s="16" t="s">
         <v>81</v>
@@ -7746,7 +7746,7 @@
         <v>34</v>
       </c>
       <c r="K91" s="19">
-        <v>120</v>
+        <v>371</v>
       </c>
       <c r="L91" s="16" t="s">
         <v>59</v>
@@ -7787,7 +7787,7 @@
         <v>30</v>
       </c>
       <c r="K92" s="19">
-        <v>549</v>
+        <v>452</v>
       </c>
       <c r="L92" s="16" t="s">
         <v>59</v>
@@ -7828,7 +7828,7 @@
         <v>32</v>
       </c>
       <c r="K93" s="19">
-        <v>251</v>
+        <v>572</v>
       </c>
       <c r="L93" s="16" t="s">
         <v>59</v>
@@ -7869,7 +7869,7 @@
         <v>34</v>
       </c>
       <c r="K94" s="19">
-        <v>410</v>
+        <v>247</v>
       </c>
       <c r="L94" s="16" t="s">
         <v>59</v>
@@ -7910,7 +7910,7 @@
         <v>32</v>
       </c>
       <c r="K95" s="19">
-        <v>288</v>
+        <v>492</v>
       </c>
       <c r="L95" s="16" t="s">
         <v>81</v>
@@ -7951,7 +7951,7 @@
         <v>34</v>
       </c>
       <c r="K96" s="19">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="L96" s="16" t="s">
         <v>59</v>
@@ -7992,7 +7992,7 @@
         <v>34</v>
       </c>
       <c r="K97" s="19">
-        <v>502</v>
+        <v>568</v>
       </c>
       <c r="L97" s="16" t="s">
         <v>81</v>
@@ -8033,7 +8033,7 @@
         <v>30</v>
       </c>
       <c r="K98" s="19">
-        <v>523</v>
+        <v>323</v>
       </c>
       <c r="L98" s="16" t="s">
         <v>59</v>
@@ -8074,7 +8074,7 @@
         <v>30</v>
       </c>
       <c r="K99" s="19">
-        <v>627</v>
+        <v>620</v>
       </c>
       <c r="L99" s="16" t="s">
         <v>59</v>
@@ -8115,7 +8115,7 @@
         <v>34</v>
       </c>
       <c r="K100" s="19">
-        <v>310</v>
+        <v>208</v>
       </c>
       <c r="L100" s="16" t="s">
         <v>59</v>
@@ -8156,7 +8156,7 @@
         <v>32</v>
       </c>
       <c r="K101" s="19">
-        <v>495</v>
+        <v>641</v>
       </c>
       <c r="L101" s="16" t="s">
         <v>59</v>
@@ -8197,7 +8197,7 @@
         <v>30</v>
       </c>
       <c r="K102" s="19">
-        <v>645</v>
+        <v>377</v>
       </c>
       <c r="L102" s="16" t="s">
         <v>59</v>
@@ -8238,7 +8238,7 @@
         <v>32</v>
       </c>
       <c r="K103" s="19">
-        <v>371</v>
+        <v>423</v>
       </c>
       <c r="L103" s="16" t="s">
         <v>59</v>
@@ -8279,7 +8279,7 @@
         <v>34</v>
       </c>
       <c r="K104" s="19">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="L104" s="16" t="s">
         <v>59</v>
@@ -8320,7 +8320,7 @@
         <v>32</v>
       </c>
       <c r="K105" s="19">
-        <v>677</v>
+        <v>323</v>
       </c>
       <c r="L105" s="16" t="s">
         <v>81</v>
@@ -8361,7 +8361,7 @@
         <v>34</v>
       </c>
       <c r="K106" s="19">
-        <v>623</v>
+        <v>424</v>
       </c>
       <c r="L106" s="16" t="s">
         <v>59</v>
@@ -8402,7 +8402,7 @@
         <v>34</v>
       </c>
       <c r="K107" s="19">
-        <v>521</v>
+        <v>510</v>
       </c>
       <c r="L107" s="16" t="s">
         <v>81</v>
@@ -8443,7 +8443,7 @@
         <v>30</v>
       </c>
       <c r="K108" s="19">
-        <v>303</v>
+        <v>232</v>
       </c>
       <c r="L108" s="16" t="s">
         <v>59</v>
@@ -8484,7 +8484,7 @@
         <v>30</v>
       </c>
       <c r="K109" s="19">
-        <v>282</v>
+        <v>328</v>
       </c>
       <c r="L109" s="16" t="s">
         <v>59</v>
@@ -8525,7 +8525,7 @@
         <v>34</v>
       </c>
       <c r="K110" s="19">
-        <v>674</v>
+        <v>345</v>
       </c>
       <c r="L110" s="16" t="s">
         <v>59</v>
@@ -8566,7 +8566,7 @@
         <v>32</v>
       </c>
       <c r="K111" s="19">
-        <v>616</v>
+        <v>527</v>
       </c>
       <c r="L111" s="16" t="s">
         <v>59</v>
@@ -8607,7 +8607,7 @@
         <v>30</v>
       </c>
       <c r="K112" s="19">
-        <v>449</v>
+        <v>637</v>
       </c>
       <c r="L112" s="16" t="s">
         <v>59</v>
@@ -8648,7 +8648,7 @@
         <v>32</v>
       </c>
       <c r="K113" s="19">
-        <v>416</v>
+        <v>234</v>
       </c>
       <c r="L113" s="16" t="s">
         <v>59</v>
@@ -8689,7 +8689,7 @@
         <v>34</v>
       </c>
       <c r="K114" s="19">
-        <v>307</v>
+        <v>480</v>
       </c>
       <c r="L114" s="16" t="s">
         <v>59</v>
@@ -8730,7 +8730,7 @@
         <v>32</v>
       </c>
       <c r="K115" s="19">
-        <v>402</v>
+        <v>641</v>
       </c>
       <c r="L115" s="16" t="s">
         <v>81</v>
@@ -8771,7 +8771,7 @@
         <v>34</v>
       </c>
       <c r="K116" s="19">
-        <v>360</v>
+        <v>333</v>
       </c>
       <c r="L116" s="16" t="s">
         <v>59</v>
@@ -8812,7 +8812,7 @@
         <v>34</v>
       </c>
       <c r="K117" s="19">
-        <v>371</v>
+        <v>237</v>
       </c>
       <c r="L117" s="16" t="s">
         <v>81</v>
@@ -8853,7 +8853,7 @@
         <v>30</v>
       </c>
       <c r="K118" s="19">
-        <v>205</v>
+        <v>642</v>
       </c>
       <c r="L118" s="16" t="s">
         <v>59</v>
@@ -8894,7 +8894,7 @@
         <v>30</v>
       </c>
       <c r="K119" s="19">
-        <v>464</v>
+        <v>644</v>
       </c>
       <c r="L119" s="16" t="s">
         <v>59</v>
@@ -8935,7 +8935,7 @@
         <v>34</v>
       </c>
       <c r="K120" s="19">
-        <v>360</v>
+        <v>234</v>
       </c>
       <c r="L120" s="16" t="s">
         <v>59</v>
@@ -8976,7 +8976,7 @@
         <v>32</v>
       </c>
       <c r="K121" s="19">
-        <v>362</v>
+        <v>663</v>
       </c>
       <c r="L121" s="16" t="s">
         <v>59</v>
@@ -9017,7 +9017,7 @@
         <v>30</v>
       </c>
       <c r="K122" s="19">
-        <v>661</v>
+        <v>306</v>
       </c>
       <c r="L122" s="16" t="s">
         <v>59</v>
@@ -9058,7 +9058,7 @@
         <v>32</v>
       </c>
       <c r="K123" s="19">
-        <v>387</v>
+        <v>534</v>
       </c>
       <c r="L123" s="16" t="s">
         <v>59</v>
@@ -9099,7 +9099,7 @@
         <v>34</v>
       </c>
       <c r="K124" s="19">
-        <v>375</v>
+        <v>553</v>
       </c>
       <c r="L124" s="16" t="s">
         <v>59</v>
@@ -9140,7 +9140,7 @@
         <v>32</v>
       </c>
       <c r="K125" s="19">
-        <v>437</v>
+        <v>317</v>
       </c>
       <c r="L125" s="16" t="s">
         <v>81</v>
@@ -9181,7 +9181,7 @@
         <v>34</v>
       </c>
       <c r="K126" s="19">
-        <v>468</v>
+        <v>625</v>
       </c>
       <c r="L126" s="16" t="s">
         <v>59</v>
@@ -9222,7 +9222,7 @@
         <v>34</v>
       </c>
       <c r="K127" s="19">
-        <v>605</v>
+        <v>280</v>
       </c>
       <c r="L127" s="16" t="s">
         <v>81</v>
@@ -9263,7 +9263,7 @@
         <v>30</v>
       </c>
       <c r="K128" s="19">
-        <v>320</v>
+        <v>698</v>
       </c>
       <c r="L128" s="16" t="s">
         <v>59</v>
@@ -9304,7 +9304,7 @@
         <v>30</v>
       </c>
       <c r="K129" s="19">
-        <v>586</v>
+        <v>604</v>
       </c>
       <c r="L129" s="16" t="s">
         <v>59</v>
@@ -9345,7 +9345,7 @@
         <v>34</v>
       </c>
       <c r="K130" s="19">
-        <v>643</v>
+        <v>285</v>
       </c>
       <c r="L130" s="16" t="s">
         <v>59</v>
@@ -9386,7 +9386,7 @@
         <v>32</v>
       </c>
       <c r="K131" s="19">
-        <v>508</v>
+        <v>629</v>
       </c>
       <c r="L131" s="16" t="s">
         <v>59</v>
@@ -9427,7 +9427,7 @@
         <v>30</v>
       </c>
       <c r="K132" s="19">
-        <v>304</v>
+        <v>525</v>
       </c>
       <c r="L132" s="16" t="s">
         <v>59</v>
@@ -9468,7 +9468,7 @@
         <v>30</v>
       </c>
       <c r="K133" s="19">
-        <v>495</v>
+        <v>280</v>
       </c>
       <c r="L133" s="16" t="s">
         <v>59</v>
@@ -9509,7 +9509,7 @@
         <v>32</v>
       </c>
       <c r="K134" s="19">
-        <v>294</v>
+        <v>538</v>
       </c>
       <c r="L134" s="16" t="s">
         <v>81</v>
@@ -9550,7 +9550,7 @@
         <v>34</v>
       </c>
       <c r="K135" s="19">
-        <v>362</v>
+        <v>622</v>
       </c>
       <c r="L135" s="16" t="s">
         <v>59</v>
@@ -9591,7 +9591,7 @@
         <v>32</v>
       </c>
       <c r="K136" s="19">
-        <v>396</v>
+        <v>543</v>
       </c>
       <c r="L136" s="16" t="s">
         <v>59</v>
@@ -9632,7 +9632,7 @@
         <v>34</v>
       </c>
       <c r="K137" s="19">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="L137" s="16" t="s">
         <v>59</v>
@@ -9673,7 +9673,7 @@
         <v>36</v>
       </c>
       <c r="K138" s="19">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="L138" s="16" t="s">
         <v>81</v>
@@ -9714,7 +9714,7 @@
         <v>30</v>
       </c>
       <c r="K139" s="19">
-        <v>394</v>
+        <v>298</v>
       </c>
       <c r="L139" s="16" t="s">
         <v>59</v>
@@ -9755,7 +9755,7 @@
         <v>32</v>
       </c>
       <c r="K140" s="19">
-        <v>519</v>
+        <v>234</v>
       </c>
       <c r="L140" s="16" t="s">
         <v>59</v>
@@ -9796,7 +9796,7 @@
         <v>34</v>
       </c>
       <c r="K141" s="19">
-        <v>499</v>
+        <v>377</v>
       </c>
       <c r="L141" s="16" t="s">
         <v>59</v>
@@ -9837,7 +9837,7 @@
         <v>32</v>
       </c>
       <c r="K142" s="19">
-        <v>459</v>
+        <v>377</v>
       </c>
       <c r="L142" s="16" t="s">
         <v>59</v>
@@ -9878,7 +9878,7 @@
         <v>32</v>
       </c>
       <c r="K143" s="19">
-        <v>472</v>
+        <v>265</v>
       </c>
       <c r="L143" s="16" t="s">
         <v>59</v>
@@ -9919,7 +9919,7 @@
         <v>36</v>
       </c>
       <c r="K144" s="19">
-        <v>375</v>
+        <v>350</v>
       </c>
       <c r="L144" s="16" t="s">
         <v>81</v>
@@ -10001,7 +10001,7 @@
         <v>32</v>
       </c>
       <c r="K146" s="19">
-        <v>270</v>
+        <v>582</v>
       </c>
       <c r="L146" s="16" t="s">
         <v>59</v>
@@ -10042,7 +10042,7 @@
         <v>30</v>
       </c>
       <c r="K147" s="19">
-        <v>192</v>
+        <v>626</v>
       </c>
       <c r="L147" s="16" t="s">
         <v>59</v>
@@ -10083,7 +10083,7 @@
         <v>30</v>
       </c>
       <c r="K148" s="19">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="L148" s="16" t="s">
         <v>59</v>
@@ -10124,7 +10124,7 @@
         <v>32</v>
       </c>
       <c r="K149" s="19">
-        <v>386</v>
+        <v>504</v>
       </c>
       <c r="L149" s="16" t="s">
         <v>81</v>
@@ -10165,7 +10165,7 @@
         <v>34</v>
       </c>
       <c r="K150" s="19">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="L150" s="16" t="s">
         <v>59</v>
@@ -10206,7 +10206,7 @@
         <v>32</v>
       </c>
       <c r="K151" s="19">
-        <v>312</v>
+        <v>265</v>
       </c>
       <c r="L151" s="16" t="s">
         <v>59</v>
@@ -10247,7 +10247,7 @@
         <v>34</v>
       </c>
       <c r="K152" s="19">
-        <v>575</v>
+        <v>396</v>
       </c>
       <c r="L152" s="16" t="s">
         <v>59</v>
@@ -10288,7 +10288,7 @@
         <v>36</v>
       </c>
       <c r="K153" s="19">
-        <v>199</v>
+        <v>336</v>
       </c>
       <c r="L153" s="16" t="s">
         <v>81</v>
@@ -10329,7 +10329,7 @@
         <v>30</v>
       </c>
       <c r="K154" s="19">
-        <v>356</v>
+        <v>227</v>
       </c>
       <c r="L154" s="16" t="s">
         <v>59</v>
@@ -10370,7 +10370,7 @@
         <v>32</v>
       </c>
       <c r="K155" s="19">
-        <v>458</v>
+        <v>543</v>
       </c>
       <c r="L155" s="16" t="s">
         <v>59</v>
@@ -10411,7 +10411,7 @@
         <v>34</v>
       </c>
       <c r="K156" s="19">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="L156" s="16" t="s">
         <v>59</v>
@@ -10452,7 +10452,7 @@
         <v>32</v>
       </c>
       <c r="K157" s="19">
-        <v>575</v>
+        <v>255</v>
       </c>
       <c r="L157" s="16" t="s">
         <v>59</v>
@@ -10493,7 +10493,7 @@
         <v>32</v>
       </c>
       <c r="K158" s="19">
-        <v>419</v>
+        <v>547</v>
       </c>
       <c r="L158" s="16" t="s">
         <v>59</v>
@@ -10534,7 +10534,7 @@
         <v>36</v>
       </c>
       <c r="K159" s="19">
-        <v>356</v>
+        <v>263</v>
       </c>
       <c r="L159" s="16" t="s">
         <v>81</v>
@@ -10575,7 +10575,7 @@
         <v>34</v>
       </c>
       <c r="K160" s="19">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="L160" s="16" t="s">
         <v>59</v>
@@ -10616,7 +10616,7 @@
         <v>32</v>
       </c>
       <c r="K161" s="19">
-        <v>258</v>
+        <v>186</v>
       </c>
       <c r="L161" s="16" t="s">
         <v>59</v>
@@ -10657,7 +10657,7 @@
         <v>30</v>
       </c>
       <c r="K162" s="19">
-        <v>618</v>
+        <v>451</v>
       </c>
       <c r="L162" s="16" t="s">
         <v>59</v>
@@ -10698,7 +10698,7 @@
         <v>30</v>
       </c>
       <c r="K163" s="19">
-        <v>439</v>
+        <v>196</v>
       </c>
       <c r="L163" s="16" t="s">
         <v>59</v>
@@ -10739,7 +10739,7 @@
         <v>32</v>
       </c>
       <c r="K164" s="19">
-        <v>251</v>
+        <v>509</v>
       </c>
       <c r="L164" s="16" t="s">
         <v>81</v>
@@ -10780,7 +10780,7 @@
         <v>34</v>
       </c>
       <c r="K165" s="19">
-        <v>422</v>
+        <v>551</v>
       </c>
       <c r="L165" s="16" t="s">
         <v>59</v>
@@ -10821,7 +10821,7 @@
         <v>32</v>
       </c>
       <c r="K166" s="19">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="L166" s="16" t="s">
         <v>59</v>
@@ -10862,7 +10862,7 @@
         <v>34</v>
       </c>
       <c r="K167" s="19">
-        <v>419</v>
+        <v>272</v>
       </c>
       <c r="L167" s="16" t="s">
         <v>59</v>
@@ -10903,7 +10903,7 @@
         <v>36</v>
       </c>
       <c r="K168" s="19">
-        <v>327</v>
+        <v>529</v>
       </c>
       <c r="L168" s="16" t="s">
         <v>81</v>
@@ -10944,7 +10944,7 @@
         <v>30</v>
       </c>
       <c r="K169" s="19">
-        <v>578</v>
+        <v>238</v>
       </c>
       <c r="L169" s="16" t="s">
         <v>59</v>
@@ -10985,7 +10985,7 @@
         <v>32</v>
       </c>
       <c r="K170" s="19">
-        <v>448</v>
+        <v>578</v>
       </c>
       <c r="L170" s="16" t="s">
         <v>59</v>
@@ -11026,7 +11026,7 @@
         <v>34</v>
       </c>
       <c r="K171" s="19">
-        <v>207</v>
+        <v>500</v>
       </c>
       <c r="L171" s="16" t="s">
         <v>59</v>
@@ -11067,7 +11067,7 @@
         <v>32</v>
       </c>
       <c r="K172" s="19">
-        <v>577</v>
+        <v>433</v>
       </c>
       <c r="L172" s="16" t="s">
         <v>59</v>
@@ -11108,7 +11108,7 @@
         <v>32</v>
       </c>
       <c r="K173" s="19">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="L173" s="16" t="s">
         <v>59</v>
@@ -11149,7 +11149,7 @@
         <v>36</v>
       </c>
       <c r="K174" s="19">
-        <v>202</v>
+        <v>278</v>
       </c>
       <c r="L174" s="16" t="s">
         <v>81</v>
@@ -11190,7 +11190,7 @@
         <v>34</v>
       </c>
       <c r="K175" s="19">
-        <v>597</v>
+        <v>440</v>
       </c>
       <c r="L175" s="16" t="s">
         <v>59</v>
@@ -11231,7 +11231,7 @@
         <v>32</v>
       </c>
       <c r="K176" s="19">
-        <v>538</v>
+        <v>356</v>
       </c>
       <c r="L176" s="16" t="s">
         <v>59</v>
@@ -11272,7 +11272,7 @@
         <v>30</v>
       </c>
       <c r="K177" s="19">
-        <v>495</v>
+        <v>192</v>
       </c>
       <c r="L177" s="16" t="s">
         <v>59</v>
@@ -11313,7 +11313,7 @@
         <v>32</v>
       </c>
       <c r="K178" s="19">
-        <v>420</v>
+        <v>478</v>
       </c>
       <c r="L178" s="16" t="s">
         <v>59</v>
@@ -11354,7 +11354,7 @@
         <v>30</v>
       </c>
       <c r="K179" s="19">
-        <v>285</v>
+        <v>246</v>
       </c>
       <c r="L179" s="16" t="s">
         <v>59</v>
@@ -11395,7 +11395,7 @@
         <v>30</v>
       </c>
       <c r="K180" s="19">
-        <v>526</v>
+        <v>192</v>
       </c>
       <c r="L180" s="16" t="s">
         <v>59</v>
@@ -11436,7 +11436,7 @@
         <v>32</v>
       </c>
       <c r="K181" s="19">
-        <v>611</v>
+        <v>219</v>
       </c>
       <c r="L181" s="16" t="s">
         <v>81</v>
@@ -11477,7 +11477,7 @@
         <v>30</v>
       </c>
       <c r="K182" s="19">
-        <v>624</v>
+        <v>282</v>
       </c>
       <c r="L182" s="16" t="s">
         <v>59</v>
@@ -11518,7 +11518,7 @@
         <v>32</v>
       </c>
       <c r="K183" s="19">
-        <v>336</v>
+        <v>596</v>
       </c>
       <c r="L183" s="16" t="s">
         <v>59</v>
@@ -11559,7 +11559,7 @@
         <v>32</v>
       </c>
       <c r="K184" s="19">
-        <v>572</v>
+        <v>187</v>
       </c>
       <c r="L184" s="16" t="s">
         <v>81</v>
@@ -11600,7 +11600,7 @@
         <v>34</v>
       </c>
       <c r="K185" s="19">
-        <v>638</v>
+        <v>173</v>
       </c>
       <c r="L185" s="16" t="s">
         <v>59</v>
@@ -11641,7 +11641,7 @@
         <v>30</v>
       </c>
       <c r="K186" s="19">
-        <v>551</v>
+        <v>266</v>
       </c>
       <c r="L186" s="16" t="s">
         <v>59</v>
@@ -11682,7 +11682,7 @@
         <v>34</v>
       </c>
       <c r="K187" s="19">
-        <v>335</v>
+        <v>236</v>
       </c>
       <c r="L187" s="16" t="s">
         <v>59</v>
@@ -11723,7 +11723,7 @@
         <v>32</v>
       </c>
       <c r="K188" s="19">
-        <v>243</v>
+        <v>480</v>
       </c>
       <c r="L188" s="16" t="s">
         <v>59</v>
@@ -11764,7 +11764,7 @@
         <v>32</v>
       </c>
       <c r="K189" s="19">
-        <v>533</v>
+        <v>260</v>
       </c>
       <c r="L189" s="16" t="s">
         <v>59</v>
@@ -11805,7 +11805,7 @@
         <v>30</v>
       </c>
       <c r="K190" s="19">
-        <v>591</v>
+        <v>608</v>
       </c>
       <c r="L190" s="16" t="s">
         <v>59</v>
@@ -11846,7 +11846,7 @@
         <v>36</v>
       </c>
       <c r="K191" s="19">
-        <v>619</v>
+        <v>180</v>
       </c>
       <c r="L191" s="16" t="s">
         <v>81</v>
@@ -11887,7 +11887,7 @@
         <v>30</v>
       </c>
       <c r="K192" s="19">
-        <v>463</v>
+        <v>636</v>
       </c>
       <c r="L192" s="16" t="s">
         <v>59</v>
@@ -11928,7 +11928,7 @@
         <v>32</v>
       </c>
       <c r="K193" s="19">
-        <v>634</v>
+        <v>596</v>
       </c>
       <c r="L193" s="16" t="s">
         <v>59</v>
@@ -11969,7 +11969,7 @@
         <v>30</v>
       </c>
       <c r="K194" s="19">
-        <v>368</v>
+        <v>242</v>
       </c>
       <c r="L194" s="16" t="s">
         <v>59</v>
@@ -12010,7 +12010,7 @@
         <v>30</v>
       </c>
       <c r="K195" s="19">
-        <v>557</v>
+        <v>617</v>
       </c>
       <c r="L195" s="16" t="s">
         <v>59</v>
@@ -12051,7 +12051,7 @@
         <v>32</v>
       </c>
       <c r="K196" s="19">
-        <v>568</v>
+        <v>302</v>
       </c>
       <c r="L196" s="16" t="s">
         <v>81</v>
@@ -12092,7 +12092,7 @@
         <v>30</v>
       </c>
       <c r="K197" s="19">
-        <v>331</v>
+        <v>532</v>
       </c>
       <c r="L197" s="16" t="s">
         <v>59</v>
@@ -12133,7 +12133,7 @@
         <v>32</v>
       </c>
       <c r="K198" s="19">
-        <v>286</v>
+        <v>563</v>
       </c>
       <c r="L198" s="16" t="s">
         <v>59</v>
@@ -12174,7 +12174,7 @@
         <v>32</v>
       </c>
       <c r="K199" s="19">
-        <v>432</v>
+        <v>350</v>
       </c>
       <c r="L199" s="16" t="s">
         <v>81</v>
@@ -12215,7 +12215,7 @@
         <v>34</v>
       </c>
       <c r="K200" s="19">
-        <v>366</v>
+        <v>563</v>
       </c>
       <c r="L200" s="16" t="s">
         <v>59</v>
@@ -12256,7 +12256,7 @@
         <v>30</v>
       </c>
       <c r="K201" s="19">
-        <v>388</v>
+        <v>547</v>
       </c>
       <c r="L201" s="16" t="s">
         <v>59</v>
@@ -12297,7 +12297,7 @@
         <v>34</v>
       </c>
       <c r="K202" s="19">
-        <v>368</v>
+        <v>501</v>
       </c>
       <c r="L202" s="16" t="s">
         <v>59</v>
@@ -12338,7 +12338,7 @@
         <v>32</v>
       </c>
       <c r="K203" s="19">
-        <v>347</v>
+        <v>495</v>
       </c>
       <c r="L203" s="16" t="s">
         <v>59</v>
@@ -12379,7 +12379,7 @@
         <v>32</v>
       </c>
       <c r="K204" s="19">
-        <v>484</v>
+        <v>464</v>
       </c>
       <c r="L204" s="16" t="s">
         <v>59</v>
@@ -12420,7 +12420,7 @@
         <v>30</v>
       </c>
       <c r="K205" s="19">
-        <v>182</v>
+        <v>408</v>
       </c>
       <c r="L205" s="16" t="s">
         <v>59</v>
@@ -12461,7 +12461,7 @@
         <v>36</v>
       </c>
       <c r="K206" s="19">
-        <v>328</v>
+        <v>615</v>
       </c>
       <c r="L206" s="16" t="s">
         <v>81</v>
@@ -12502,7 +12502,7 @@
         <v>30</v>
       </c>
       <c r="K207" s="19">
-        <v>239</v>
+        <v>289</v>
       </c>
       <c r="L207" s="16" t="s">
         <v>59</v>
@@ -12543,7 +12543,7 @@
         <v>32</v>
       </c>
       <c r="K208" s="19">
-        <v>280</v>
+        <v>400</v>
       </c>
       <c r="L208" s="16" t="s">
         <v>59</v>
@@ -12584,7 +12584,7 @@
         <v>30</v>
       </c>
       <c r="K209" s="19">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="L209" s="16" t="s">
         <v>59</v>
@@ -12625,7 +12625,7 @@
         <v>30</v>
       </c>
       <c r="K210" s="19">
-        <v>332</v>
+        <v>166</v>
       </c>
       <c r="L210" s="16" t="s">
         <v>59</v>
@@ -12666,7 +12666,7 @@
         <v>32</v>
       </c>
       <c r="K211" s="19">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="L211" s="16" t="s">
         <v>81</v>
@@ -12707,7 +12707,7 @@
         <v>30</v>
       </c>
       <c r="K212" s="19">
-        <v>183</v>
+        <v>433</v>
       </c>
       <c r="L212" s="16" t="s">
         <v>59</v>
@@ -12748,7 +12748,7 @@
         <v>32</v>
       </c>
       <c r="K213" s="19">
-        <v>290</v>
+        <v>200</v>
       </c>
       <c r="L213" s="16" t="s">
         <v>59</v>
@@ -12789,7 +12789,7 @@
         <v>32</v>
       </c>
       <c r="K214" s="19">
-        <v>493</v>
+        <v>275</v>
       </c>
       <c r="L214" s="16" t="s">
         <v>81</v>
@@ -12830,7 +12830,7 @@
         <v>34</v>
       </c>
       <c r="K215" s="19">
-        <v>250</v>
+        <v>308</v>
       </c>
       <c r="L215" s="16" t="s">
         <v>59</v>
@@ -12871,7 +12871,7 @@
         <v>30</v>
       </c>
       <c r="K216" s="19">
-        <v>554</v>
+        <v>585</v>
       </c>
       <c r="L216" s="16" t="s">
         <v>59</v>
@@ -12912,7 +12912,7 @@
         <v>34</v>
       </c>
       <c r="K217" s="19">
-        <v>279</v>
+        <v>630</v>
       </c>
       <c r="L217" s="16" t="s">
         <v>59</v>
@@ -12953,7 +12953,7 @@
         <v>32</v>
       </c>
       <c r="K218" s="19">
-        <v>215</v>
+        <v>353</v>
       </c>
       <c r="L218" s="16" t="s">
         <v>59</v>
@@ -12994,7 +12994,7 @@
         <v>32</v>
       </c>
       <c r="K219" s="19">
-        <v>295</v>
+        <v>495</v>
       </c>
       <c r="L219" s="16" t="s">
         <v>59</v>
@@ -13035,7 +13035,7 @@
         <v>30</v>
       </c>
       <c r="K220" s="19">
-        <v>590</v>
+        <v>240</v>
       </c>
       <c r="L220" s="16" t="s">
         <v>59</v>
@@ -13076,7 +13076,7 @@
         <v>36</v>
       </c>
       <c r="K221" s="19">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="L221" s="16" t="s">
         <v>81</v>
@@ -13117,7 +13117,7 @@
         <v>30</v>
       </c>
       <c r="K222" s="19">
-        <v>355</v>
+        <v>301</v>
       </c>
       <c r="L222" s="16" t="s">
         <v>59</v>
@@ -13158,7 +13158,7 @@
         <v>30</v>
       </c>
       <c r="K223" s="19">
-        <v>192</v>
+        <v>241</v>
       </c>
       <c r="L223" s="16" t="s">
         <v>59</v>
@@ -13199,7 +13199,7 @@
         <v>32</v>
       </c>
       <c r="K224" s="19">
-        <v>247</v>
+        <v>224</v>
       </c>
       <c r="L224" s="16" t="s">
         <v>59</v>
@@ -13240,7 +13240,7 @@
         <v>30</v>
       </c>
       <c r="K225" s="19">
-        <v>400</v>
+        <v>462</v>
       </c>
       <c r="L225" s="16" t="s">
         <v>59</v>
@@ -13281,7 +13281,7 @@
         <v>34</v>
       </c>
       <c r="K226" s="19">
-        <v>378</v>
+        <v>477</v>
       </c>
       <c r="L226" s="16" t="s">
         <v>81</v>
@@ -13322,7 +13322,7 @@
         <v>32</v>
       </c>
       <c r="K227" s="19">
-        <v>498</v>
+        <v>141</v>
       </c>
       <c r="L227" s="16" t="s">
         <v>59</v>
@@ -13363,7 +13363,7 @@
         <v>34</v>
       </c>
       <c r="K228" s="19">
-        <v>305</v>
+        <v>369</v>
       </c>
       <c r="L228" s="16" t="s">
         <v>59</v>
@@ -13404,7 +13404,7 @@
         <v>30</v>
       </c>
       <c r="K229" s="19">
-        <v>506</v>
+        <v>366</v>
       </c>
       <c r="L229" s="16" t="s">
         <v>59</v>
@@ -13445,7 +13445,7 @@
         <v>32</v>
       </c>
       <c r="K230" s="19">
-        <v>473</v>
+        <v>423</v>
       </c>
       <c r="L230" s="16" t="s">
         <v>59</v>
@@ -13486,7 +13486,7 @@
         <v>32</v>
       </c>
       <c r="K231" s="19">
-        <v>221</v>
+        <v>357</v>
       </c>
       <c r="L231" s="16" t="s">
         <v>59</v>
@@ -13527,7 +13527,7 @@
         <v>34</v>
       </c>
       <c r="K232" s="19">
-        <v>235</v>
+        <v>253</v>
       </c>
       <c r="L232" s="16" t="s">
         <v>81</v>
@@ -13568,7 +13568,7 @@
         <v>36</v>
       </c>
       <c r="K233" s="19">
-        <v>402</v>
+        <v>516</v>
       </c>
       <c r="L233" s="16" t="s">
         <v>59</v>
@@ -13609,7 +13609,7 @@
         <v>30</v>
       </c>
       <c r="K234" s="19">
-        <v>370</v>
+        <v>454</v>
       </c>
       <c r="L234" s="16" t="s">
         <v>59</v>
@@ -13650,7 +13650,7 @@
         <v>36</v>
       </c>
       <c r="K235" s="19">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="L235" s="16" t="s">
         <v>59</v>
@@ -13691,7 +13691,7 @@
         <v>32</v>
       </c>
       <c r="K236" s="19">
-        <v>257</v>
+        <v>348</v>
       </c>
       <c r="L236" s="16" t="s">
         <v>59</v>
@@ -13732,7 +13732,7 @@
         <v>30</v>
       </c>
       <c r="K237" s="19">
-        <v>266</v>
+        <v>455</v>
       </c>
       <c r="L237" s="16" t="s">
         <v>59</v>
@@ -13773,7 +13773,7 @@
         <v>30</v>
       </c>
       <c r="K238" s="19">
-        <v>340</v>
+        <v>191</v>
       </c>
       <c r="L238" s="16" t="s">
         <v>59</v>
@@ -13814,7 +13814,7 @@
         <v>32</v>
       </c>
       <c r="K239" s="19">
-        <v>503</v>
+        <v>385</v>
       </c>
       <c r="L239" s="16" t="s">
         <v>59</v>
@@ -13855,7 +13855,7 @@
         <v>30</v>
       </c>
       <c r="K240" s="19">
-        <v>550</v>
+        <v>144</v>
       </c>
       <c r="L240" s="16" t="s">
         <v>59</v>
@@ -13896,7 +13896,7 @@
         <v>34</v>
       </c>
       <c r="K241" s="19">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="L241" s="16" t="s">
         <v>81</v>
@@ -13937,7 +13937,7 @@
         <v>32</v>
       </c>
       <c r="K242" s="19">
-        <v>159</v>
+        <v>209</v>
       </c>
       <c r="L242" s="16" t="s">
         <v>59</v>
@@ -13978,7 +13978,7 @@
         <v>34</v>
       </c>
       <c r="K243" s="19">
-        <v>491</v>
+        <v>306</v>
       </c>
       <c r="L243" s="16" t="s">
         <v>59</v>
@@ -14019,7 +14019,7 @@
         <v>30</v>
       </c>
       <c r="K244" s="19">
-        <v>351</v>
+        <v>223</v>
       </c>
       <c r="L244" s="16" t="s">
         <v>59</v>
@@ -14060,7 +14060,7 @@
         <v>32</v>
       </c>
       <c r="K245" s="19">
-        <v>357</v>
+        <v>178</v>
       </c>
       <c r="L245" s="16" t="s">
         <v>59</v>
@@ -14101,7 +14101,7 @@
         <v>32</v>
       </c>
       <c r="K246" s="19">
-        <v>176</v>
+        <v>260</v>
       </c>
       <c r="L246" s="16" t="s">
         <v>59</v>
@@ -14142,7 +14142,7 @@
         <v>34</v>
       </c>
       <c r="K247" s="19">
-        <v>510</v>
+        <v>393</v>
       </c>
       <c r="L247" s="16" t="s">
         <v>81</v>
@@ -14183,7 +14183,7 @@
         <v>36</v>
       </c>
       <c r="K248" s="19">
-        <v>183</v>
+        <v>514</v>
       </c>
       <c r="L248" s="16" t="s">
         <v>59</v>
@@ -14224,7 +14224,7 @@
         <v>30</v>
       </c>
       <c r="K249" s="19">
-        <v>343</v>
+        <v>142</v>
       </c>
       <c r="L249" s="16" t="s">
         <v>59</v>
@@ -14265,7 +14265,7 @@
         <v>36</v>
       </c>
       <c r="K250" s="19">
-        <v>207</v>
+        <v>513</v>
       </c>
       <c r="L250" s="16" t="s">
         <v>59</v>
@@ -14306,7 +14306,7 @@
         <v>32</v>
       </c>
       <c r="K251" s="19">
-        <v>264</v>
+        <v>397</v>
       </c>
       <c r="L251" s="16" t="s">
         <v>59</v>
@@ -14347,7 +14347,7 @@
         <v>30</v>
       </c>
       <c r="K252" s="19">
-        <v>161</v>
+        <v>457</v>
       </c>
       <c r="L252" s="16" t="s">
         <v>59</v>
@@ -14388,7 +14388,7 @@
         <v>30</v>
       </c>
       <c r="K253" s="19">
-        <v>521</v>
+        <v>240</v>
       </c>
       <c r="L253" s="16" t="s">
         <v>59</v>
@@ -14429,7 +14429,7 @@
         <v>32</v>
       </c>
       <c r="K254" s="19">
-        <v>180</v>
+        <v>433</v>
       </c>
       <c r="L254" s="16" t="s">
         <v>59</v>
@@ -14470,7 +14470,7 @@
         <v>30</v>
       </c>
       <c r="K255" s="19">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="L255" s="16" t="s">
         <v>59</v>
@@ -14511,7 +14511,7 @@
         <v>34</v>
       </c>
       <c r="K256" s="19">
-        <v>489</v>
+        <v>442</v>
       </c>
       <c r="L256" s="16" t="s">
         <v>81</v>
@@ -14552,7 +14552,7 @@
         <v>32</v>
       </c>
       <c r="K257" s="19">
-        <v>337</v>
+        <v>207</v>
       </c>
       <c r="L257" s="16" t="s">
         <v>59</v>
@@ -14593,7 +14593,7 @@
         <v>34</v>
       </c>
       <c r="K258" s="19">
-        <v>150</v>
+        <v>323</v>
       </c>
       <c r="L258" s="16" t="s">
         <v>59</v>
@@ -14634,7 +14634,7 @@
         <v>30</v>
       </c>
       <c r="K259" s="19">
-        <v>500</v>
+        <v>558</v>
       </c>
       <c r="L259" s="16" t="s">
         <v>59</v>
@@ -14675,7 +14675,7 @@
         <v>32</v>
       </c>
       <c r="K260" s="19">
-        <v>171</v>
+        <v>357</v>
       </c>
       <c r="L260" s="16" t="s">
         <v>59</v>
@@ -14716,7 +14716,7 @@
         <v>32</v>
       </c>
       <c r="K261" s="19">
-        <v>325</v>
+        <v>304</v>
       </c>
       <c r="L261" s="16" t="s">
         <v>59</v>
@@ -14757,7 +14757,7 @@
         <v>34</v>
       </c>
       <c r="K262" s="19">
-        <v>407</v>
+        <v>367</v>
       </c>
       <c r="L262" s="16" t="s">
         <v>81</v>
@@ -14798,7 +14798,7 @@
         <v>36</v>
       </c>
       <c r="K263" s="19">
-        <v>349</v>
+        <v>184</v>
       </c>
       <c r="L263" s="16" t="s">
         <v>59</v>
@@ -14839,7 +14839,7 @@
         <v>30</v>
       </c>
       <c r="K264" s="19">
-        <v>438</v>
+        <v>272</v>
       </c>
       <c r="L264" s="16" t="s">
         <v>59</v>
@@ -14880,7 +14880,7 @@
         <v>36</v>
       </c>
       <c r="K265" s="19">
-        <v>503</v>
+        <v>188</v>
       </c>
       <c r="L265" s="16" t="s">
         <v>59</v>
@@ -14921,7 +14921,7 @@
         <v>32</v>
       </c>
       <c r="K266" s="19">
-        <v>300</v>
+        <v>517</v>
       </c>
       <c r="L266" s="16" t="s">
         <v>59</v>
@@ -14962,7 +14962,7 @@
         <v>32</v>
       </c>
       <c r="K267" s="19">
-        <v>337</v>
+        <v>481</v>
       </c>
       <c r="L267" s="16" t="s">
         <v>59</v>
@@ -15003,7 +15003,7 @@
         <v>36</v>
       </c>
       <c r="K268" s="19">
-        <v>137</v>
+        <v>436</v>
       </c>
       <c r="L268" s="16" t="s">
         <v>81</v>
@@ -15044,7 +15044,7 @@
         <v>36</v>
       </c>
       <c r="K269" s="19">
-        <v>158</v>
+        <v>459</v>
       </c>
       <c r="L269" s="16" t="s">
         <v>59</v>
@@ -15085,7 +15085,7 @@
         <v>30</v>
       </c>
       <c r="K270" s="19">
-        <v>262</v>
+        <v>463</v>
       </c>
       <c r="L270" s="16" t="s">
         <v>59</v>
@@ -15126,7 +15126,7 @@
         <v>34</v>
       </c>
       <c r="K271" s="19">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L271" s="16" t="s">
         <v>59</v>
@@ -15167,7 +15167,7 @@
         <v>34</v>
       </c>
       <c r="K272" s="19">
-        <v>441</v>
+        <v>308</v>
       </c>
       <c r="L272" s="16" t="s">
         <v>59</v>
@@ -15208,7 +15208,7 @@
         <v>36</v>
       </c>
       <c r="K273" s="19">
-        <v>393</v>
+        <v>201</v>
       </c>
       <c r="L273" s="16" t="s">
         <v>59</v>
@@ -15249,7 +15249,7 @@
         <v>30</v>
       </c>
       <c r="K274" s="19">
-        <v>400</v>
+        <v>266</v>
       </c>
       <c r="L274" s="16" t="s">
         <v>59</v>
@@ -15290,7 +15290,7 @@
         <v>32</v>
       </c>
       <c r="K275" s="19">
-        <v>289</v>
+        <v>347</v>
       </c>
       <c r="L275" s="16" t="s">
         <v>59</v>
@@ -15331,7 +15331,7 @@
         <v>32</v>
       </c>
       <c r="K276" s="19">
-        <v>289</v>
+        <v>445</v>
       </c>
       <c r="L276" s="16" t="s">
         <v>59</v>
@@ -15372,7 +15372,7 @@
         <v>32</v>
       </c>
       <c r="K277" s="19">
-        <v>491</v>
+        <v>443</v>
       </c>
       <c r="L277" s="16" t="s">
         <v>59</v>
@@ -15413,7 +15413,7 @@
         <v>36</v>
       </c>
       <c r="K278" s="19">
-        <v>239</v>
+        <v>212</v>
       </c>
       <c r="L278" s="16" t="s">
         <v>81</v>
@@ -15454,7 +15454,7 @@
         <v>36</v>
       </c>
       <c r="K279" s="19">
-        <v>372</v>
+        <v>418</v>
       </c>
       <c r="L279" s="16" t="s">
         <v>59</v>
@@ -15495,7 +15495,7 @@
         <v>30</v>
       </c>
       <c r="K280" s="19">
-        <v>397</v>
+        <v>333</v>
       </c>
       <c r="L280" s="16" t="s">
         <v>59</v>
@@ -15536,7 +15536,7 @@
         <v>34</v>
       </c>
       <c r="K281" s="19">
-        <v>290</v>
+        <v>180</v>
       </c>
       <c r="L281" s="16" t="s">
         <v>59</v>
@@ -15577,7 +15577,7 @@
         <v>34</v>
       </c>
       <c r="K282" s="19">
-        <v>415</v>
+        <v>324</v>
       </c>
       <c r="L282" s="16" t="s">
         <v>59</v>
@@ -15618,7 +15618,7 @@
         <v>36</v>
       </c>
       <c r="K283" s="19">
-        <v>471</v>
+        <v>167</v>
       </c>
       <c r="L283" s="16" t="s">
         <v>59</v>
@@ -15659,7 +15659,7 @@
         <v>30</v>
       </c>
       <c r="K284" s="19">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="L284" s="16" t="s">
         <v>59</v>
@@ -15700,7 +15700,7 @@
         <v>32</v>
       </c>
       <c r="K285" s="19">
-        <v>397</v>
+        <v>283</v>
       </c>
       <c r="L285" s="16" t="s">
         <v>59</v>
@@ -15741,7 +15741,7 @@
         <v>32</v>
       </c>
       <c r="K286" s="19">
-        <v>483</v>
+        <v>461</v>
       </c>
       <c r="L286" s="16" t="s">
         <v>59</v>
@@ -15782,7 +15782,7 @@
         <v>32</v>
       </c>
       <c r="K287" s="19">
-        <v>245</v>
+        <v>500</v>
       </c>
       <c r="L287" s="16" t="s">
         <v>59</v>
@@ -15823,7 +15823,7 @@
         <v>36</v>
       </c>
       <c r="K288" s="19">
-        <v>202</v>
+        <v>437</v>
       </c>
       <c r="L288" s="16" t="s">
         <v>81</v>
@@ -15864,7 +15864,7 @@
         <v>36</v>
       </c>
       <c r="K289" s="19">
-        <v>271</v>
+        <v>288</v>
       </c>
       <c r="L289" s="16" t="s">
         <v>59</v>
@@ -15905,7 +15905,7 @@
         <v>30</v>
       </c>
       <c r="K290" s="19">
-        <v>280</v>
+        <v>310</v>
       </c>
       <c r="L290" s="16" t="s">
         <v>59</v>
@@ -15946,7 +15946,7 @@
         <v>34</v>
       </c>
       <c r="K291" s="19">
-        <v>172</v>
+        <v>502</v>
       </c>
       <c r="L291" s="16" t="s">
         <v>59</v>
@@ -15987,7 +15987,7 @@
         <v>34</v>
       </c>
       <c r="K292" s="19">
-        <v>164</v>
+        <v>219</v>
       </c>
       <c r="L292" s="16" t="s">
         <v>59</v>
@@ -16028,7 +16028,7 @@
         <v>36</v>
       </c>
       <c r="K293" s="19">
-        <v>468</v>
+        <v>285</v>
       </c>
       <c r="L293" s="16" t="s">
         <v>59</v>
@@ -16069,7 +16069,7 @@
         <v>30</v>
       </c>
       <c r="K294" s="19">
-        <v>409</v>
+        <v>451</v>
       </c>
       <c r="L294" s="16" t="s">
         <v>59</v>
@@ -16110,7 +16110,7 @@
         <v>32</v>
       </c>
       <c r="K295" s="19">
-        <v>347</v>
+        <v>130</v>
       </c>
       <c r="L295" s="16" t="s">
         <v>59</v>
@@ -16151,7 +16151,7 @@
         <v>32</v>
       </c>
       <c r="K296" s="19">
-        <v>455</v>
+        <v>211</v>
       </c>
       <c r="L296" s="16" t="s">
         <v>59</v>
@@ -16192,7 +16192,7 @@
         <v>32</v>
       </c>
       <c r="K297" s="19">
-        <v>313</v>
+        <v>438</v>
       </c>
       <c r="L297" s="16" t="s">
         <v>59</v>
@@ -16233,7 +16233,7 @@
         <v>36</v>
       </c>
       <c r="K298" s="19">
-        <v>401</v>
+        <v>263</v>
       </c>
       <c r="L298" s="16" t="s">
         <v>81</v>
@@ -16274,7 +16274,7 @@
         <v>36</v>
       </c>
       <c r="K299" s="19">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="L299" s="16" t="s">
         <v>59</v>
@@ -16315,7 +16315,7 @@
         <v>30</v>
       </c>
       <c r="K300" s="19">
-        <v>453</v>
+        <v>494</v>
       </c>
       <c r="L300" s="16" t="s">
         <v>59</v>
@@ -16356,7 +16356,7 @@
         <v>34</v>
       </c>
       <c r="K301" s="19">
-        <v>227</v>
+        <v>493</v>
       </c>
       <c r="L301" s="16" t="s">
         <v>59</v>
@@ -16397,7 +16397,7 @@
         <v>34</v>
       </c>
       <c r="K302" s="19">
-        <v>381</v>
+        <v>242</v>
       </c>
       <c r="L302" s="16" t="s">
         <v>59</v>
@@ -16438,7 +16438,7 @@
         <v>36</v>
       </c>
       <c r="K303" s="19">
-        <v>494</v>
+        <v>356</v>
       </c>
       <c r="L303" s="16" t="s">
         <v>59</v>
@@ -16479,7 +16479,7 @@
         <v>30</v>
       </c>
       <c r="K304" s="19">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="L304" s="16" t="s">
         <v>59</v>
@@ -16520,7 +16520,7 @@
         <v>32</v>
       </c>
       <c r="K305" s="19">
-        <v>401</v>
+        <v>420</v>
       </c>
       <c r="L305" s="16" t="s">
         <v>59</v>
@@ -16561,7 +16561,7 @@
         <v>32</v>
       </c>
       <c r="K306" s="19">
-        <v>381</v>
+        <v>134</v>
       </c>
       <c r="L306" s="16" t="s">
         <v>59</v>
@@ -16602,7 +16602,7 @@
         <v>32</v>
       </c>
       <c r="K307" s="19">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="L307" s="16" t="s">
         <v>59</v>
@@ -16643,7 +16643,7 @@
         <v>36</v>
       </c>
       <c r="K308" s="19">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="L308" s="16" t="s">
         <v>81</v>
@@ -16684,7 +16684,7 @@
         <v>36</v>
       </c>
       <c r="K309" s="19">
-        <v>374</v>
+        <v>139</v>
       </c>
       <c r="L309" s="16" t="s">
         <v>59</v>
@@ -16725,7 +16725,7 @@
         <v>30</v>
       </c>
       <c r="K310" s="19">
-        <v>261</v>
+        <v>389</v>
       </c>
       <c r="L310" s="16" t="s">
         <v>59</v>
@@ -16766,7 +16766,7 @@
         <v>34</v>
       </c>
       <c r="K311" s="19">
-        <v>232</v>
+        <v>197</v>
       </c>
       <c r="L311" s="16" t="s">
         <v>59</v>
@@ -16807,7 +16807,7 @@
         <v>34</v>
       </c>
       <c r="K312" s="19">
-        <v>134</v>
+        <v>406</v>
       </c>
       <c r="L312" s="16" t="s">
         <v>59</v>
@@ -16848,7 +16848,7 @@
         <v>36</v>
       </c>
       <c r="K313" s="19">
-        <v>334</v>
+        <v>362</v>
       </c>
       <c r="L313" s="16" t="s">
         <v>59</v>
@@ -16889,7 +16889,7 @@
         <v>30</v>
       </c>
       <c r="K314" s="19">
-        <v>302</v>
+        <v>193</v>
       </c>
       <c r="L314" s="16" t="s">
         <v>59</v>
@@ -16930,7 +16930,7 @@
         <v>32</v>
       </c>
       <c r="K315" s="19">
-        <v>131</v>
+        <v>290</v>
       </c>
       <c r="L315" s="16" t="s">
         <v>59</v>
@@ -16971,7 +16971,7 @@
         <v>32</v>
       </c>
       <c r="K316" s="19">
-        <v>265</v>
+        <v>337</v>
       </c>
       <c r="L316" s="16" t="s">
         <v>59</v>
@@ -17012,7 +17012,7 @@
         <v>30</v>
       </c>
       <c r="K317" s="19">
-        <v>289</v>
+        <v>184</v>
       </c>
       <c r="L317" s="16" t="s">
         <v>81</v>
@@ -17053,7 +17053,7 @@
         <v>30</v>
       </c>
       <c r="K318" s="19">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="L318" s="16" t="s">
         <v>59</v>
@@ -17094,7 +17094,7 @@
         <v>32</v>
       </c>
       <c r="K319" s="19">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="L319" s="16" t="s">
         <v>59</v>
@@ -17135,7 +17135,7 @@
         <v>30</v>
       </c>
       <c r="K320" s="19">
-        <v>417</v>
+        <v>292</v>
       </c>
       <c r="L320" s="16" t="s">
         <v>59</v>
@@ -17176,7 +17176,7 @@
         <v>30</v>
       </c>
       <c r="K321" s="19">
-        <v>201</v>
+        <v>112</v>
       </c>
       <c r="L321" s="16" t="s">
         <v>59</v>
@@ -17217,7 +17217,7 @@
         <v>32</v>
       </c>
       <c r="K322" s="19">
-        <v>204</v>
+        <v>386</v>
       </c>
       <c r="L322" s="16" t="s">
         <v>59</v>
@@ -17258,7 +17258,7 @@
         <v>34</v>
       </c>
       <c r="K323" s="19">
-        <v>234</v>
+        <v>348</v>
       </c>
       <c r="L323" s="16" t="s">
         <v>81</v>
@@ -17299,7 +17299,7 @@
         <v>32</v>
       </c>
       <c r="K324" s="19">
-        <v>163</v>
+        <v>411</v>
       </c>
       <c r="L324" s="16" t="s">
         <v>59</v>
@@ -17340,7 +17340,7 @@
         <v>34</v>
       </c>
       <c r="K325" s="19">
-        <v>237</v>
+        <v>164</v>
       </c>
       <c r="L325" s="16" t="s">
         <v>59</v>
@@ -17381,7 +17381,7 @@
         <v>34</v>
       </c>
       <c r="K326" s="19">
-        <v>331</v>
+        <v>249</v>
       </c>
       <c r="L326" s="16" t="s">
         <v>59</v>
@@ -17422,7 +17422,7 @@
         <v>30</v>
       </c>
       <c r="K327" s="19">
-        <v>302</v>
+        <v>397</v>
       </c>
       <c r="L327" s="16" t="s">
         <v>81</v>
@@ -17463,7 +17463,7 @@
         <v>30</v>
       </c>
       <c r="K328" s="19">
-        <v>320</v>
+        <v>413</v>
       </c>
       <c r="L328" s="16" t="s">
         <v>59</v>
@@ -17504,7 +17504,7 @@
         <v>32</v>
       </c>
       <c r="K329" s="19">
-        <v>302</v>
+        <v>233</v>
       </c>
       <c r="L329" s="16" t="s">
         <v>59</v>
@@ -17545,7 +17545,7 @@
         <v>30</v>
       </c>
       <c r="K330" s="19">
-        <v>375</v>
+        <v>226</v>
       </c>
       <c r="L330" s="16" t="s">
         <v>59</v>
@@ -17586,7 +17586,7 @@
         <v>30</v>
       </c>
       <c r="K331" s="19">
-        <v>254</v>
+        <v>289</v>
       </c>
       <c r="L331" s="16" t="s">
         <v>59</v>
@@ -17627,7 +17627,7 @@
         <v>32</v>
       </c>
       <c r="K332" s="19">
-        <v>302</v>
+        <v>174</v>
       </c>
       <c r="L332" s="16" t="s">
         <v>59</v>
@@ -17668,7 +17668,7 @@
         <v>34</v>
       </c>
       <c r="K333" s="19">
-        <v>387</v>
+        <v>190</v>
       </c>
       <c r="L333" s="16" t="s">
         <v>81</v>
@@ -17709,7 +17709,7 @@
         <v>32</v>
       </c>
       <c r="K334" s="19">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="L334" s="16" t="s">
         <v>59</v>
@@ -17750,7 +17750,7 @@
         <v>34</v>
       </c>
       <c r="K335" s="19">
-        <v>115</v>
+        <v>183</v>
       </c>
       <c r="L335" s="16" t="s">
         <v>59</v>
@@ -17791,7 +17791,7 @@
         <v>34</v>
       </c>
       <c r="K336" s="19">
-        <v>359</v>
+        <v>290</v>
       </c>
       <c r="L336" s="16" t="s">
         <v>59</v>
@@ -17832,7 +17832,7 @@
         <v>30</v>
       </c>
       <c r="K337" s="19">
-        <v>254</v>
+        <v>132</v>
       </c>
       <c r="L337" s="16" t="s">
         <v>81</v>
@@ -17873,7 +17873,7 @@
         <v>30</v>
       </c>
       <c r="K338" s="19">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="L338" s="16" t="s">
         <v>59</v>
@@ -17914,7 +17914,7 @@
         <v>32</v>
       </c>
       <c r="K339" s="19">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="L339" s="16" t="s">
         <v>59</v>
@@ -17955,7 +17955,7 @@
         <v>30</v>
       </c>
       <c r="K340" s="19">
-        <v>337</v>
+        <v>143</v>
       </c>
       <c r="L340" s="16" t="s">
         <v>59</v>
@@ -17996,7 +17996,7 @@
         <v>30</v>
       </c>
       <c r="K341" s="19">
-        <v>241</v>
+        <v>290</v>
       </c>
       <c r="L341" s="16" t="s">
         <v>59</v>
@@ -18037,7 +18037,7 @@
         <v>32</v>
       </c>
       <c r="K342" s="19">
-        <v>429</v>
+        <v>138</v>
       </c>
       <c r="L342" s="16" t="s">
         <v>59</v>
@@ -18078,7 +18078,7 @@
         <v>34</v>
       </c>
       <c r="K343" s="19">
-        <v>278</v>
+        <v>218</v>
       </c>
       <c r="L343" s="16" t="s">
         <v>81</v>
@@ -18119,7 +18119,7 @@
         <v>32</v>
       </c>
       <c r="K344" s="19">
-        <v>421</v>
+        <v>341</v>
       </c>
       <c r="L344" s="16" t="s">
         <v>59</v>
@@ -18160,7 +18160,7 @@
         <v>34</v>
       </c>
       <c r="K345" s="19">
-        <v>360</v>
+        <v>130</v>
       </c>
       <c r="L345" s="16" t="s">
         <v>59</v>
@@ -18201,7 +18201,7 @@
         <v>34</v>
       </c>
       <c r="K346" s="19">
-        <v>401</v>
+        <v>160</v>
       </c>
       <c r="L346" s="16" t="s">
         <v>59</v>
@@ -18242,7 +18242,7 @@
         <v>30</v>
       </c>
       <c r="K347" s="19">
-        <v>130</v>
+        <v>415</v>
       </c>
       <c r="L347" s="16" t="s">
         <v>81</v>
@@ -18283,7 +18283,7 @@
         <v>30</v>
       </c>
       <c r="K348" s="19">
-        <v>359</v>
+        <v>310</v>
       </c>
       <c r="L348" s="16" t="s">
         <v>59</v>
@@ -18324,7 +18324,7 @@
         <v>32</v>
       </c>
       <c r="K349" s="19">
-        <v>377</v>
+        <v>208</v>
       </c>
       <c r="L349" s="16" t="s">
         <v>59</v>
@@ -18365,7 +18365,7 @@
         <v>30</v>
       </c>
       <c r="K350" s="19">
-        <v>417</v>
+        <v>351</v>
       </c>
       <c r="L350" s="16" t="s">
         <v>59</v>
@@ -18406,7 +18406,7 @@
         <v>30</v>
       </c>
       <c r="K351" s="19">
-        <v>386</v>
+        <v>259</v>
       </c>
       <c r="L351" s="16" t="s">
         <v>59</v>
@@ -18447,7 +18447,7 @@
         <v>32</v>
       </c>
       <c r="K352" s="19">
-        <v>113</v>
+        <v>384</v>
       </c>
       <c r="L352" s="16" t="s">
         <v>59</v>
@@ -18488,7 +18488,7 @@
         <v>34</v>
       </c>
       <c r="K353" s="19">
-        <v>114</v>
+        <v>423</v>
       </c>
       <c r="L353" s="16" t="s">
         <v>81</v>
@@ -18529,7 +18529,7 @@
         <v>32</v>
       </c>
       <c r="K354" s="19">
-        <v>216</v>
+        <v>139</v>
       </c>
       <c r="L354" s="16" t="s">
         <v>59</v>
@@ -18570,7 +18570,7 @@
         <v>34</v>
       </c>
       <c r="K355" s="19">
-        <v>189</v>
+        <v>281</v>
       </c>
       <c r="L355" s="16" t="s">
         <v>59</v>
@@ -18611,7 +18611,7 @@
         <v>34</v>
       </c>
       <c r="K356" s="19">
-        <v>387</v>
+        <v>281</v>
       </c>
       <c r="L356" s="16" t="s">
         <v>59</v>
@@ -18652,7 +18652,7 @@
         <v>30</v>
       </c>
       <c r="K357" s="19">
-        <v>371</v>
+        <v>130</v>
       </c>
       <c r="L357" s="16" t="s">
         <v>81</v>
@@ -18693,7 +18693,7 @@
         <v>30</v>
       </c>
       <c r="K358" s="19">
-        <v>388</v>
+        <v>417</v>
       </c>
       <c r="L358" s="16" t="s">
         <v>59</v>
@@ -18734,7 +18734,7 @@
         <v>32</v>
       </c>
       <c r="K359" s="19">
-        <v>214</v>
+        <v>256</v>
       </c>
       <c r="L359" s="16" t="s">
         <v>59</v>
@@ -18775,7 +18775,7 @@
         <v>30</v>
       </c>
       <c r="K360" s="19">
-        <v>341</v>
+        <v>233</v>
       </c>
       <c r="L360" s="16" t="s">
         <v>59</v>
@@ -18816,7 +18816,7 @@
         <v>30</v>
       </c>
       <c r="K361" s="19">
-        <v>247</v>
+        <v>194</v>
       </c>
       <c r="L361" s="16" t="s">
         <v>59</v>
@@ -18857,7 +18857,7 @@
         <v>32</v>
       </c>
       <c r="K362" s="19">
-        <v>330</v>
+        <v>278</v>
       </c>
       <c r="L362" s="16" t="s">
         <v>59</v>
@@ -18898,7 +18898,7 @@
         <v>34</v>
       </c>
       <c r="K363" s="19">
-        <v>142</v>
+        <v>370</v>
       </c>
       <c r="L363" s="16" t="s">
         <v>81</v>
@@ -18939,7 +18939,7 @@
         <v>32</v>
       </c>
       <c r="K364" s="19">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="L364" s="16" t="s">
         <v>59</v>
@@ -18980,7 +18980,7 @@
         <v>34</v>
       </c>
       <c r="K365" s="19">
-        <v>272</v>
+        <v>369</v>
       </c>
       <c r="L365" s="16" t="s">
         <v>59</v>
@@ -19021,7 +19021,7 @@
         <v>34</v>
       </c>
       <c r="K366" s="19">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="L366" s="16" t="s">
         <v>59</v>

</xml_diff>